<commit_message>
Fix speed, reliability, and heading-position bugs
</commit_message>
<xml_diff>
--- a/Item_Master_Enriched.xlsx
+++ b/Item_Master_Enriched.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\COA System\coa_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E9C4DE8-DC41-49B4-BCA2-B17BBCB19860}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A919FA40-ABBA-4E5B-A3D1-A237E1E40A2C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>